<commit_message>
Backup QR Scanner data - 2026-03-17T11:17:14.581Z - Cache Bust: 1773746234581
</commit_message>
<xml_diff>
--- a/log_history/Y5_B2627_Nephrology_scanner1773674746428_1cbef68ff1c1ac113f1f1ad07d544e6bd59f1108d6b7404b7db2c14564e46c2b.xlsx
+++ b/log_history/Y5_B2627_Nephrology_scanner1773674746428_1cbef68ff1c1ac113f1f1ad07d544e6bd59f1108d6b7404b7db2c14564e46c2b.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Nephrology" sheetId="1" r:id="rId1"/>
+    <sheet name="Scanner" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1279,9 +1279,29 @@
         <v>asunephrologyresident@gmail.com</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>211604</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Nephrology</v>
+      </c>
+      <c r="C45" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="D45" t="str">
+        <v>13:16:24</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F45" t="str">
+        <v>asunephrologyresident@gmail.com</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>